<commit_message>
Upload Equipment Ball Mill.xlsx via Zeta Client
</commit_message>
<xml_diff>
--- a/EQUIPMENT/Equipment Ball Mill.xlsx
+++ b/EQUIPMENT/Equipment Ball Mill.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hamxi\Documents\Zeta_Edit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99C795A0-95B2-4EF3-AE29-684379DE749A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98A6EF41-FDC4-4D9E-B85C-9A53AE3CB25C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{D2660FC1-993F-477B-80D5-6A27395D5F63}"/>
   </bookViews>
   <sheets>
     <sheet name="FLOW METER CALCULATION" sheetId="1" r:id="rId1"/>
-    <sheet name="PERANCANGAN (CONCEPT &amp; DESIGN)" sheetId="2" r:id="rId2"/>
+    <sheet name="PERANCANGAN  (CONCEPT &amp; DESIGN)" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -530,6 +530,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -563,7 +564,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1636,16 +1636,16 @@
   <sheetData>
     <row r="2" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="23"/>
-      <c r="D3" s="24"/>
-      <c r="F3" s="22" t="s">
+      <c r="C3" s="24"/>
+      <c r="D3" s="25"/>
+      <c r="F3" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="23"/>
-      <c r="H3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="25"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
@@ -1775,10 +1775,10 @@
       <c r="D11" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="25" t="s">
+      <c r="F11" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="G11" s="26"/>
+      <c r="G11" s="27"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
@@ -1864,22 +1864,22 @@
       <c r="G17" s="4"/>
     </row>
     <row r="18" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="J18" s="19" t="s">
+      <c r="J18" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="K18" s="20"/>
-      <c r="L18" s="20"/>
-      <c r="M18" s="20"/>
-      <c r="N18" s="20"/>
-      <c r="O18" s="21"/>
+      <c r="K18" s="21"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="21"/>
+      <c r="O18" s="22"/>
     </row>
     <row r="19" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="20" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="C20" s="23"/>
-      <c r="D20" s="24"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="25"/>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B21" s="1" t="s">
@@ -2048,21 +2048,21 @@
     </row>
     <row r="39" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="40" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="27" t="s">
+      <c r="B40" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="C40" s="28"/>
-      <c r="D40" s="29"/>
+      <c r="C40" s="29"/>
+      <c r="D40" s="30"/>
     </row>
     <row r="41" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="J41" s="19" t="s">
+      <c r="J41" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="K41" s="20"/>
-      <c r="L41" s="20"/>
-      <c r="M41" s="20"/>
-      <c r="N41" s="20"/>
-      <c r="O41" s="21"/>
+      <c r="K41" s="21"/>
+      <c r="L41" s="21"/>
+      <c r="M41" s="21"/>
+      <c r="N41" s="21"/>
+      <c r="O41" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2091,7 +2091,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="4" spans="4:4" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="D4" s="30" t="s">
+      <c r="D4" s="19" t="s">
         <v>80</v>
       </c>
     </row>

</xml_diff>